<commit_message>
Polish language support - v2.3.2
</commit_message>
<xml_diff>
--- a/translations.xlsx
+++ b/translations.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\peter\Documents\vscode\homebridge-gree-airconditioner\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/peter/VSCode/homebridge-gree-airconditioner/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34F1380E-FEC8-4516-B4F5-07210AB5D350}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70B53600-C945-804D-97C8-FA9EDFEF2D72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{12A545F6-ED01-499F-B40F-8257FFC4F2F0}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="36600" windowHeight="21260" xr2:uid="{12A545F6-ED01-499F-B40F-8257FFC4F2F0}"/>
   </bookViews>
   <sheets>
     <sheet name="config.schema.json" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="445">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="584" uniqueCount="517">
   <si>
     <t>Key</t>
   </si>
@@ -848,9 +848,6 @@
     <t>Fűtés/hűtés módban használt függőleges lamellapozíció</t>
   </si>
   <si>
-    <t>Vertical swing position to be used in heating/cooling modes</t>
-  </si>
-  <si>
     <t>Ventilátorüzemmód-vezérlés engedélyezve</t>
   </si>
   <si>
@@ -1371,6 +1368,225 @@
   </si>
   <si>
     <t>Posición de oscilación vertical para el modo ventilador</t>
+  </si>
+  <si>
+    <t>disableBroadcast.title</t>
+  </si>
+  <si>
+    <t>disableBroadcast.description</t>
+  </si>
+  <si>
+    <t>Disable broadcast</t>
+  </si>
+  <si>
+    <t>If broadcast is disabled, only unicast messages are sent on the network</t>
+  </si>
+  <si>
+    <t>Vertical swing position to be set in heating/cooling modes</t>
+  </si>
+  <si>
+    <t>Polish</t>
+  </si>
+  <si>
+    <t>pl</t>
+  </si>
+  <si>
+    <t>Model z 3 stopniami prędkości</t>
+  </si>
+  <si>
+    <t>Model z 5 stopniami prędkości</t>
+  </si>
+  <si>
+    <t>Wyłączony</t>
+  </si>
+  <si>
+    <t>Akcesorium podrzędne</t>
+  </si>
+  <si>
+    <t>Akcesorium oddzielne</t>
+  </si>
+  <si>
+    <t>Nigdy</t>
+  </si>
+  <si>
+    <t>Zastępuj ustawienia domyślne po włączeniu urządzenia</t>
+  </si>
+  <si>
+    <t>Zastępuj ustawienia domyślne po włączeniu urządzenia lub wyłączeniu oscylowania</t>
+  </si>
+  <si>
+    <t>Ustawiaj zawsze po włączeniu urządzenia</t>
+  </si>
+  <si>
+    <t>Ustawiaj zawsze po włączeniu urządzenia lub wyłączeniu trybu oscylowania</t>
+  </si>
+  <si>
+    <t>Domyślna dla urządzenia</t>
+  </si>
+  <si>
+    <t>Stała – najwyższa</t>
+  </si>
+  <si>
+    <t>Stała – wyższa</t>
+  </si>
+  <si>
+    <t>Stała – środkowa</t>
+  </si>
+  <si>
+    <t>Stała – niższa</t>
+  </si>
+  <si>
+    <t>Stała – najniższa</t>
+  </si>
+  <si>
+    <t>Automatyczny</t>
+  </si>
+  <si>
+    <t>Nazwa:</t>
+  </si>
+  <si>
+    <t>Port UDP na poziomie bridge używany do wykrywania urządzeń (automatyczny, jeśli pole puste)</t>
+  </si>
+  <si>
+    <t>Odstęp czasowy skanowania:</t>
+  </si>
+  <si>
+    <t>Odstęp czasowy między próbami wykrycia urządzenia (60 sekund, jeśli pole puste)</t>
+  </si>
+  <si>
+    <t>Wyłącz automatyczne wykrywanie</t>
+  </si>
+  <si>
+    <t>Gdy automatycznie wykrywanie jest wyłączone, jedynie jednostki wpisane w sekcji Urządzenia będą aktywne</t>
+  </si>
+  <si>
+    <t>Wyłącz tryb broadcast</t>
+  </si>
+  <si>
+    <t>Gdy tryb broadcast jest wyłączony, wyłącznie komunikaty unicast będą wysyłane w sieci</t>
+  </si>
+  <si>
+    <t>Urządzenia</t>
+  </si>
+  <si>
+    <t>Dodaj urządzenie</t>
+  </si>
+  <si>
+    <t>Adres MAC (numer seryjny):</t>
+  </si>
+  <si>
+    <t>Adres MAC urządzenia (małe litery, bez seperatorów)&lt;br /&gt;LUB&lt;br /&gt;wartość specjalna: &lt;b&gt;domyślna&lt;/b&gt;</t>
+  </si>
+  <si>
+    <t>Nazwa urządzenia:</t>
+  </si>
+  <si>
+    <t>Własna nazwa urządzenia. Używaj wyłącznie znaków alfanumerycznych, spacji i apostrofu. Upewnij się, że zaczyna się i kończy znakiem alfanumerycznym. Unikaj emoji.</t>
+  </si>
+  <si>
+    <t>Dezaktywuj urządzenie</t>
+  </si>
+  <si>
+    <t>Jeśli pole jest zaznaczone, urządzenie zostanie usunięte z usługi HomeKit, oraz będzie przez nią ignorowane</t>
+  </si>
+  <si>
+    <t>Adres IP:</t>
+  </si>
+  <si>
+    <t>Adres IP urządzenia (automatyczny, jeśli pole puste)</t>
+  </si>
+  <si>
+    <t>Port UDP dedykowany dla urządzenia (automatyczny, jeśli pole puste)</t>
+  </si>
+  <si>
+    <t>Odstęp między zmianami statusu:</t>
+  </si>
+  <si>
+    <t>Odstęp między aktualizacjami statusu urządzenia (w sekundach)</t>
+  </si>
+  <si>
+    <t>Poziom szyfrowania protokołu sieciowego:</t>
+  </si>
+  <si>
+    <t>Pozostaw automatyczny. Jeśli nie działa, ustaw konkretną wersję.</t>
+  </si>
+  <si>
+    <t>Model urządzenia:</t>
+  </si>
+  <si>
+    <t>Poziomy prędkości wentylatora:</t>
+  </si>
+  <si>
+    <t>Minimalna wartość temperatury docelowej:</t>
+  </si>
+  <si>
+    <t>Minimalna wartość temperatury docelowej (w ℃)</t>
+  </si>
+  <si>
+    <t>Maksymalna wartość temperatury docelowej:</t>
+  </si>
+  <si>
+    <t>Maksymalna wartość temperatury docelowej (w ℃)</t>
+  </si>
+  <si>
+    <t>Przesunięcie temperatury:</t>
+  </si>
+  <si>
+    <t>Korekta czujnika temperatury (w ℃)</t>
+  </si>
+  <si>
+    <t>Różnica stopni temperatur:</t>
+  </si>
+  <si>
+    <t>Poprawne wartości: 0.5 (dla °F) oraz 1 (dla °C)&lt;BR /&gt;(Liczenie z parametru jednostek temperatury Homebridge UI jeśli pusty lub nieprawidłowy)</t>
+  </si>
+  <si>
+    <t>Włącz xFan</t>
+  </si>
+  <si>
+    <t>Jeśli aktywny, funkcja xFan będzie włączana automatycznie</t>
+  </si>
+  <si>
+    <t>Czujnik temperatury:</t>
+  </si>
+  <si>
+    <t>Dodatkowy czujnik temperatury w aplikacji HomeKit</t>
+  </si>
+  <si>
+    <t>Modyfikuj pionową pozycję skrzydła:</t>
+  </si>
+  <si>
+    <t>Wybierz, kiedy pionowa pozycja skrzydła ma być modyfikowana</t>
+  </si>
+  <si>
+    <t>Pionowa pozycja skrzydła:</t>
+  </si>
+  <si>
+    <t>Pionowa pozycja skrzydła w trybach grzania/chłodzenia</t>
+  </si>
+  <si>
+    <t>Włącz kontrolę wentylatora</t>
+  </si>
+  <si>
+    <t>Jeśli funkcja aktywna, kontrola wentylatora zostanie dodana do aplikacji Dom a obsługa trybu wentylatora włączona</t>
+  </si>
+  <si>
+    <t>Pionowa pozycja skrzydła w trybie wentylatora:</t>
+  </si>
+  <si>
+    <t>Pionowa pozycja skrzydła, która ma być ustawiona w trybie wentylatora</t>
+  </si>
+  <si>
+    <t>Zakres czasowy trybu cichego:</t>
+  </si>
+  <si>
+    <t>Godziny, w których jednostka nie powinna piszczeć przy wydawaniu jej poleceń (format: HH:MM-HH:MM, np.: 22:00-08:30)</t>
+  </si>
+  <si>
+    <t>Broadcast kikapcsolása</t>
+  </si>
+  <si>
+    <t>Ha a broadcast ki van kapcsolva, csak unicast üzeneteket küld a rendszer a hálózaton</t>
   </si>
 </sst>
 </file>
@@ -1785,19 +2001,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38CF4BE7-6125-49FF-9193-D3853B48D530}">
-  <dimension ref="A1:G72"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:H74"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="35.42578125" customWidth="1"/>
-    <col min="2" max="2" width="51.85546875" customWidth="1"/>
-    <col min="3" max="3" width="11.7109375" customWidth="1"/>
-    <col min="4" max="4" width="11.28515625" customWidth="1"/>
-    <col min="5" max="5" width="8.85546875" customWidth="1"/>
-    <col min="6" max="6" width="12.85546875" customWidth="1"/>
-    <col min="7" max="7" width="21.85546875" customWidth="1"/>
+    <col min="1" max="1" width="35.5" customWidth="1"/>
+    <col min="2" max="2" width="51.83203125" customWidth="1"/>
+    <col min="3" max="3" width="11.6640625" customWidth="1"/>
+    <col min="4" max="4" width="11.33203125" customWidth="1"/>
+    <col min="5" max="5" width="8.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1819,8 +2035,11 @@
       <c r="G1" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H1" s="2" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -1842,8 +2061,11 @@
       <c r="G2" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H2" s="1" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -1854,7 +2076,7 @@
         <v>236</v>
       </c>
       <c r="D3" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="E3" t="s">
         <v>144</v>
@@ -1865,8 +2087,11 @@
       <c r="G3" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H3" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>15</v>
       </c>
@@ -1877,7 +2102,7 @@
         <v>235</v>
       </c>
       <c r="D4" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="E4" t="s">
         <v>145</v>
@@ -1888,8 +2113,11 @@
       <c r="G4" t="s">
         <v>147</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H4" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -1911,8 +2139,11 @@
       <c r="G5" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H5" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>17</v>
       </c>
@@ -1923,19 +2154,22 @@
         <v>237</v>
       </c>
       <c r="D6" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="E6" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="F6" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="G6" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+        <v>359</v>
+      </c>
+      <c r="H6" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>18</v>
       </c>
@@ -1946,19 +2180,22 @@
         <v>238</v>
       </c>
       <c r="D7" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="E7" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="F7" t="s">
         <v>153</v>
       </c>
       <c r="G7" t="s">
-        <v>361</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+        <v>360</v>
+      </c>
+      <c r="H7" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>22</v>
       </c>
@@ -1980,8 +2217,11 @@
       <c r="G8" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H8" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>23</v>
       </c>
@@ -1992,19 +2232,22 @@
         <v>158</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E9" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="F9" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="G9" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H9" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>24</v>
       </c>
@@ -2015,19 +2258,22 @@
         <v>239</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="E10" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="F10" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="G10" t="s">
-        <v>362</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+        <v>361</v>
+      </c>
+      <c r="H10" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -2038,19 +2284,22 @@
         <v>159</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="F11" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="G11" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H11" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>26</v>
       </c>
@@ -2061,19 +2310,22 @@
         <v>240</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="F12" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="G12" t="s">
-        <v>363</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+        <v>362</v>
+      </c>
+      <c r="H12" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>32</v>
       </c>
@@ -2084,19 +2336,22 @@
         <v>241</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="F13" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="G13" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H13" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>33</v>
       </c>
@@ -2107,19 +2362,22 @@
         <v>242</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="E14" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="F14" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="G14" t="s">
-        <v>364</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+        <v>363</v>
+      </c>
+      <c r="H14" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>34</v>
       </c>
@@ -2130,19 +2388,22 @@
         <v>243</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="E15" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="F15" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="G15" t="s">
-        <v>365</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+        <v>364</v>
+      </c>
+      <c r="H15" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>35</v>
       </c>
@@ -2153,19 +2414,22 @@
         <v>244</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="E16" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="F16" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="G16" t="s">
-        <v>366</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+        <v>365</v>
+      </c>
+      <c r="H16" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>36</v>
       </c>
@@ -2176,19 +2440,22 @@
         <v>245</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="E17" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="F17" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="G17" t="s">
-        <v>367</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+        <v>366</v>
+      </c>
+      <c r="H17" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>37</v>
       </c>
@@ -2199,19 +2466,22 @@
         <v>246</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="E18" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="F18" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="G18" t="s">
-        <v>368</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+        <v>367</v>
+      </c>
+      <c r="H18" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>44</v>
       </c>
@@ -2222,19 +2492,22 @@
         <v>241</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="F19" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="G19" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H19" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>45</v>
       </c>
@@ -2245,19 +2518,22 @@
         <v>242</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="E20" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="F20" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="G20" t="s">
-        <v>364</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+        <v>363</v>
+      </c>
+      <c r="H20" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>46</v>
       </c>
@@ -2268,19 +2544,22 @@
         <v>243</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="E21" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="F21" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="G21" t="s">
-        <v>365</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+        <v>364</v>
+      </c>
+      <c r="H21" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>47</v>
       </c>
@@ -2291,19 +2570,22 @@
         <v>244</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="E22" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="F22" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="G22" t="s">
-        <v>366</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+        <v>365</v>
+      </c>
+      <c r="H22" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>48</v>
       </c>
@@ -2314,19 +2596,22 @@
         <v>245</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="E23" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="F23" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="G23" t="s">
-        <v>367</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+        <v>366</v>
+      </c>
+      <c r="H23" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>49</v>
       </c>
@@ -2337,19 +2622,22 @@
         <v>246</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="E24" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="F24" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="G24" t="s">
-        <v>368</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+        <v>367</v>
+      </c>
+      <c r="H24" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>50</v>
       </c>
@@ -2371,15 +2659,18 @@
       <c r="G25" t="s">
         <v>166</v>
       </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H25" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>54</v>
       </c>
-      <c r="B26" s="3" t="s">
+      <c r="B26" t="s">
         <v>52</v>
       </c>
-      <c r="C26" s="3" t="s">
+      <c r="C26" t="s">
         <v>167</v>
       </c>
       <c r="D26" s="3" t="s">
@@ -2394,15 +2685,18 @@
       <c r="G26" s="3" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H26" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>55</v>
       </c>
-      <c r="B27" s="3" t="s">
+      <c r="B27" t="s">
         <v>53</v>
       </c>
-      <c r="C27" s="3" t="s">
+      <c r="C27" t="s">
         <v>53</v>
       </c>
       <c r="D27" s="3" t="s">
@@ -2417,8 +2711,11 @@
       <c r="G27" s="3" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H27" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>56</v>
       </c>
@@ -2429,42 +2726,48 @@
         <v>247</v>
       </c>
       <c r="D28" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="E28" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="F28" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>419</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+        <v>418</v>
+      </c>
+      <c r="H28" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>57</v>
       </c>
-      <c r="B29" s="3" t="s">
+      <c r="B29" t="s">
         <v>59</v>
       </c>
-      <c r="C29" s="3" t="s">
+      <c r="C29" t="s">
         <v>248</v>
       </c>
       <c r="D29" s="3" t="s">
         <v>174</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>369</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+        <v>368</v>
+      </c>
+      <c r="H29" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>58</v>
       </c>
@@ -2475,19 +2778,22 @@
         <v>249</v>
       </c>
       <c r="D30" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="F30" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="G30" t="s">
-        <v>370</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+        <v>369</v>
+      </c>
+      <c r="H30" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>61</v>
       </c>
@@ -2504,13 +2810,16 @@
         <v>176</v>
       </c>
       <c r="F31" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="G31" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H31" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>62</v>
       </c>
@@ -2521,936 +2830,1087 @@
         <v>251</v>
       </c>
       <c r="D32" t="s">
+        <v>280</v>
+      </c>
+      <c r="E32" t="s">
+        <v>311</v>
+      </c>
+      <c r="F32" t="s">
+        <v>338</v>
+      </c>
+      <c r="G32" t="s">
+        <v>370</v>
+      </c>
+      <c r="H32" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>444</v>
+      </c>
+      <c r="B33" t="s">
+        <v>446</v>
+      </c>
+      <c r="C33" t="s">
+        <v>515</v>
+      </c>
+      <c r="H33" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>445</v>
+      </c>
+      <c r="B34" t="s">
+        <v>447</v>
+      </c>
+      <c r="C34" t="s">
+        <v>516</v>
+      </c>
+      <c r="H34" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>65</v>
+      </c>
+      <c r="B35" t="s">
+        <v>67</v>
+      </c>
+      <c r="C35" t="s">
+        <v>181</v>
+      </c>
+      <c r="D35" t="s">
+        <v>180</v>
+      </c>
+      <c r="E35" t="s">
+        <v>179</v>
+      </c>
+      <c r="F35" t="s">
+        <v>178</v>
+      </c>
+      <c r="G35" t="s">
+        <v>178</v>
+      </c>
+      <c r="H35" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>66</v>
+      </c>
+      <c r="B36" t="s">
+        <v>68</v>
+      </c>
+      <c r="C36" t="s">
+        <v>182</v>
+      </c>
+      <c r="D36" t="s">
+        <v>183</v>
+      </c>
+      <c r="E36" t="s">
+        <v>184</v>
+      </c>
+      <c r="F36" t="s">
+        <v>185</v>
+      </c>
+      <c r="G36" t="s">
+        <v>186</v>
+      </c>
+      <c r="H36" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>71</v>
+      </c>
+      <c r="B37" t="s">
+        <v>69</v>
+      </c>
+      <c r="C37" t="s">
+        <v>187</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="E37" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="F37" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="G37" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="H37" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>72</v>
+      </c>
+      <c r="B38" t="s">
+        <v>70</v>
+      </c>
+      <c r="C38" t="s">
+        <v>252</v>
+      </c>
+      <c r="D38" t="s">
         <v>281</v>
       </c>
-      <c r="E32" t="s">
+      <c r="E38" t="s">
         <v>312</v>
       </c>
-      <c r="F32" t="s">
+      <c r="F38" t="s">
         <v>339</v>
       </c>
-      <c r="G32" t="s">
+      <c r="G38" t="s">
         <v>371</v>
       </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>65</v>
-      </c>
-      <c r="B33" t="s">
-        <v>67</v>
-      </c>
-      <c r="C33" t="s">
-        <v>181</v>
-      </c>
-      <c r="D33" t="s">
-        <v>180</v>
-      </c>
-      <c r="E33" t="s">
-        <v>179</v>
-      </c>
-      <c r="F33" t="s">
-        <v>178</v>
-      </c>
-      <c r="G33" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>66</v>
-      </c>
-      <c r="B34" t="s">
-        <v>68</v>
-      </c>
-      <c r="C34" t="s">
-        <v>182</v>
-      </c>
-      <c r="D34" t="s">
-        <v>183</v>
-      </c>
-      <c r="E34" t="s">
-        <v>184</v>
-      </c>
-      <c r="F34" t="s">
-        <v>185</v>
-      </c>
-      <c r="G34" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>71</v>
-      </c>
-      <c r="B35" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="C35" s="3" t="s">
-        <v>187</v>
-      </c>
-      <c r="D35" s="3" t="s">
-        <v>189</v>
-      </c>
-      <c r="E35" s="3" t="s">
-        <v>198</v>
-      </c>
-      <c r="F35" s="3" t="s">
-        <v>191</v>
-      </c>
-      <c r="G35" s="3" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>72</v>
-      </c>
-      <c r="B36" t="s">
-        <v>70</v>
-      </c>
-      <c r="C36" t="s">
-        <v>252</v>
-      </c>
-      <c r="D36" t="s">
+      <c r="H38" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>73</v>
+      </c>
+      <c r="B39" t="s">
+        <v>75</v>
+      </c>
+      <c r="C39" t="s">
+        <v>188</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="E39" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="F39" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="G39" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="H39" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>74</v>
+      </c>
+      <c r="B40" t="s">
+        <v>76</v>
+      </c>
+      <c r="C40" t="s">
+        <v>253</v>
+      </c>
+      <c r="D40" s="4" t="s">
+        <v>428</v>
+      </c>
+      <c r="E40" s="4" t="s">
+        <v>403</v>
+      </c>
+      <c r="F40" t="s">
+        <v>392</v>
+      </c>
+      <c r="G40" t="s">
+        <v>393</v>
+      </c>
+      <c r="H40" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>77</v>
+      </c>
+      <c r="B41" t="s">
+        <v>19</v>
+      </c>
+      <c r="C41" t="s">
+        <v>151</v>
+      </c>
+      <c r="D41" t="s">
+        <v>150</v>
+      </c>
+      <c r="E41" t="s">
+        <v>152</v>
+      </c>
+      <c r="F41" t="s">
+        <v>149</v>
+      </c>
+      <c r="G41" t="s">
+        <v>148</v>
+      </c>
+      <c r="H41" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>78</v>
+      </c>
+      <c r="B42" t="s">
+        <v>79</v>
+      </c>
+      <c r="C42" t="s">
+        <v>254</v>
+      </c>
+      <c r="D42" t="s">
         <v>282</v>
       </c>
-      <c r="E36" t="s">
-        <v>313</v>
-      </c>
-      <c r="F36" t="s">
+      <c r="E42" t="s">
+        <v>314</v>
+      </c>
+      <c r="F42" t="s">
         <v>340</v>
       </c>
-      <c r="G36" t="s">
+      <c r="G42" t="s">
         <v>372</v>
       </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>73</v>
-      </c>
-      <c r="B37" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="C37" s="3" t="s">
-        <v>188</v>
-      </c>
-      <c r="D37" s="3" t="s">
-        <v>190</v>
-      </c>
-      <c r="E37" s="3" t="s">
-        <v>314</v>
-      </c>
-      <c r="F37" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="G37" s="3" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>74</v>
-      </c>
-      <c r="B38" t="s">
-        <v>76</v>
-      </c>
-      <c r="C38" t="s">
-        <v>253</v>
-      </c>
-      <c r="D38" s="4" t="s">
+      <c r="H42" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>80</v>
+      </c>
+      <c r="B43" t="s">
+        <v>82</v>
+      </c>
+      <c r="C43" t="s">
+        <v>195</v>
+      </c>
+      <c r="D43" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="E43" s="3" t="s">
+        <v>197</v>
+      </c>
+      <c r="F43" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="G43" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="H43" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>81</v>
+      </c>
+      <c r="B44" t="s">
+        <v>83</v>
+      </c>
+      <c r="C44" t="s">
+        <v>255</v>
+      </c>
+      <c r="D44" s="4" t="s">
         <v>429</v>
       </c>
-      <c r="E38" s="4" t="s">
+      <c r="E44" t="s">
+        <v>199</v>
+      </c>
+      <c r="F44" t="s">
+        <v>201</v>
+      </c>
+      <c r="G44" t="s">
+        <v>204</v>
+      </c>
+      <c r="H44" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>85</v>
+      </c>
+      <c r="B45" t="s">
+        <v>53</v>
+      </c>
+      <c r="C45" t="s">
+        <v>53</v>
+      </c>
+      <c r="D45" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="E45" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="F45" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="G45" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="H45" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>86</v>
+      </c>
+      <c r="B46" t="s">
+        <v>84</v>
+      </c>
+      <c r="C46" t="s">
+        <v>256</v>
+      </c>
+      <c r="D46" t="s">
+        <v>283</v>
+      </c>
+      <c r="E46" s="4" t="s">
         <v>404</v>
       </c>
-      <c r="F38" t="s">
-        <v>393</v>
-      </c>
-      <c r="G38" t="s">
+      <c r="F46" t="s">
+        <v>202</v>
+      </c>
+      <c r="G46" t="s">
+        <v>205</v>
+      </c>
+      <c r="H46" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>87</v>
+      </c>
+      <c r="B47" t="s">
+        <v>89</v>
+      </c>
+      <c r="C47" t="s">
+        <v>206</v>
+      </c>
+      <c r="D47" s="3" t="s">
+        <v>284</v>
+      </c>
+      <c r="E47" s="4" t="s">
+        <v>405</v>
+      </c>
+      <c r="F47" s="3" t="s">
+        <v>341</v>
+      </c>
+      <c r="G47" s="3" t="s">
+        <v>373</v>
+      </c>
+      <c r="H47" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>88</v>
+      </c>
+      <c r="B48" t="s">
+        <v>90</v>
+      </c>
+      <c r="C48" t="s">
+        <v>257</v>
+      </c>
+      <c r="D48" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="E48" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="F48" s="4" t="s">
+        <v>440</v>
+      </c>
+      <c r="G48" t="s">
+        <v>374</v>
+      </c>
+      <c r="H48" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>91</v>
+      </c>
+      <c r="B49" t="s">
+        <v>93</v>
+      </c>
+      <c r="C49" t="s">
+        <v>258</v>
+      </c>
+      <c r="D49" s="3" t="s">
+        <v>285</v>
+      </c>
+      <c r="E49" s="4" t="s">
+        <v>407</v>
+      </c>
+      <c r="F49" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="G49" s="3" t="s">
+        <v>208</v>
+      </c>
+      <c r="H49" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>92</v>
+      </c>
+      <c r="B50" t="s">
+        <v>94</v>
+      </c>
+      <c r="C50" t="s">
+        <v>259</v>
+      </c>
+      <c r="D50" t="s">
+        <v>286</v>
+      </c>
+      <c r="E50" s="4" t="s">
+        <v>408</v>
+      </c>
+      <c r="F50" t="s">
+        <v>342</v>
+      </c>
+      <c r="G50" t="s">
+        <v>375</v>
+      </c>
+      <c r="H50" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>95</v>
+      </c>
+      <c r="B51" t="s">
+        <v>96</v>
+      </c>
+      <c r="C51" t="s">
+        <v>209</v>
+      </c>
+      <c r="D51" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="E51" s="3" t="s">
+        <v>315</v>
+      </c>
+      <c r="F51" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="G51" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="H51" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>97</v>
+      </c>
+      <c r="B52" t="s">
+        <v>98</v>
+      </c>
+      <c r="C52" t="s">
+        <v>260</v>
+      </c>
+      <c r="D52" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="E52" s="4" t="s">
+        <v>417</v>
+      </c>
+      <c r="F52" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="G52" s="3" t="s">
+        <v>376</v>
+      </c>
+      <c r="H52" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>99</v>
+      </c>
+      <c r="B53" t="s">
+        <v>101</v>
+      </c>
+      <c r="C53" t="s">
+        <v>214</v>
+      </c>
+      <c r="D53" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="E53" s="4" t="s">
+        <v>409</v>
+      </c>
+      <c r="F53" s="3" t="s">
+        <v>343</v>
+      </c>
+      <c r="G53" s="3" t="s">
+        <v>377</v>
+      </c>
+      <c r="H53" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
+        <v>100</v>
+      </c>
+      <c r="B54" t="s">
+        <v>102</v>
+      </c>
+      <c r="C54" t="s">
+        <v>261</v>
+      </c>
+      <c r="D54" t="s">
+        <v>289</v>
+      </c>
+      <c r="E54" s="4" t="s">
+        <v>410</v>
+      </c>
+      <c r="F54" t="s">
+        <v>344</v>
+      </c>
+      <c r="G54" t="s">
+        <v>378</v>
+      </c>
+      <c r="H54" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
+        <v>103</v>
+      </c>
+      <c r="B55" t="s">
+        <v>105</v>
+      </c>
+      <c r="C55" t="s">
+        <v>215</v>
+      </c>
+      <c r="D55" s="3" t="s">
+        <v>290</v>
+      </c>
+      <c r="E55" s="4" t="s">
+        <v>411</v>
+      </c>
+      <c r="F55" s="3" t="s">
+        <v>345</v>
+      </c>
+      <c r="G55" s="3" t="s">
+        <v>379</v>
+      </c>
+      <c r="H55" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
+        <v>104</v>
+      </c>
+      <c r="B56" t="s">
+        <v>106</v>
+      </c>
+      <c r="C56" t="s">
+        <v>262</v>
+      </c>
+      <c r="D56" t="s">
+        <v>291</v>
+      </c>
+      <c r="E56" s="4" t="s">
+        <v>412</v>
+      </c>
+      <c r="F56" t="s">
+        <v>346</v>
+      </c>
+      <c r="G56" t="s">
+        <v>380</v>
+      </c>
+      <c r="H56" t="s">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
+        <v>109</v>
+      </c>
+      <c r="B57" t="s">
+        <v>107</v>
+      </c>
+      <c r="C57" t="s">
+        <v>263</v>
+      </c>
+      <c r="D57" s="3" t="s">
+        <v>292</v>
+      </c>
+      <c r="E57" s="3" t="s">
+        <v>316</v>
+      </c>
+      <c r="F57" s="3" t="s">
+        <v>347</v>
+      </c>
+      <c r="G57" s="3" t="s">
+        <v>347</v>
+      </c>
+      <c r="H57" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
+        <v>110</v>
+      </c>
+      <c r="B58" t="s">
+        <v>108</v>
+      </c>
+      <c r="C58" t="s">
+        <v>264</v>
+      </c>
+      <c r="D58" t="s">
+        <v>293</v>
+      </c>
+      <c r="E58" t="s">
+        <v>317</v>
+      </c>
+      <c r="F58" t="s">
+        <v>348</v>
+      </c>
+      <c r="G58" t="s">
+        <v>381</v>
+      </c>
+      <c r="H58" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
+        <v>111</v>
+      </c>
+      <c r="B59" t="s">
+        <v>113</v>
+      </c>
+      <c r="C59" t="s">
+        <v>265</v>
+      </c>
+      <c r="D59" s="4" t="s">
+        <v>431</v>
+      </c>
+      <c r="E59" s="3" t="s">
+        <v>318</v>
+      </c>
+      <c r="F59" s="3" t="s">
+        <v>216</v>
+      </c>
+      <c r="G59" s="3" t="s">
+        <v>216</v>
+      </c>
+      <c r="H59" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A60" t="s">
+        <v>112</v>
+      </c>
+      <c r="B60" t="s">
+        <v>114</v>
+      </c>
+      <c r="C60" t="s">
+        <v>349</v>
+      </c>
+      <c r="D60" s="4" t="s">
+        <v>432</v>
+      </c>
+      <c r="E60" t="s">
+        <v>350</v>
+      </c>
+      <c r="F60" t="s">
+        <v>351</v>
+      </c>
+      <c r="G60" t="s">
+        <v>382</v>
+      </c>
+      <c r="H60" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A61" t="s">
+        <v>115</v>
+      </c>
+      <c r="B61" t="s">
+        <v>117</v>
+      </c>
+      <c r="C61" t="s">
+        <v>217</v>
+      </c>
+      <c r="D61" t="s">
+        <v>395</v>
+      </c>
+      <c r="E61" t="s">
+        <v>218</v>
+      </c>
+      <c r="F61" t="s">
+        <v>352</v>
+      </c>
+      <c r="G61" t="s">
+        <v>398</v>
+      </c>
+      <c r="H61" t="s">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A62" t="s">
+        <v>116</v>
+      </c>
+      <c r="B62" t="s">
+        <v>118</v>
+      </c>
+      <c r="C62" t="s">
+        <v>266</v>
+      </c>
+      <c r="D62" t="s">
         <v>394</v>
       </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>77</v>
-      </c>
-      <c r="B39" t="s">
-        <v>19</v>
-      </c>
-      <c r="C39" t="s">
-        <v>151</v>
-      </c>
-      <c r="D39" t="s">
-        <v>150</v>
-      </c>
-      <c r="E39" t="s">
-        <v>152</v>
-      </c>
-      <c r="F39" t="s">
-        <v>149</v>
-      </c>
-      <c r="G39" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>78</v>
-      </c>
-      <c r="B40" t="s">
-        <v>79</v>
-      </c>
-      <c r="C40" t="s">
-        <v>254</v>
-      </c>
-      <c r="D40" t="s">
-        <v>283</v>
-      </c>
-      <c r="E40" t="s">
-        <v>315</v>
-      </c>
-      <c r="F40" t="s">
-        <v>341</v>
-      </c>
-      <c r="G40" t="s">
-        <v>373</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
-        <v>80</v>
-      </c>
-      <c r="B41" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="C41" s="3" t="s">
-        <v>195</v>
-      </c>
-      <c r="D41" s="3" t="s">
-        <v>196</v>
-      </c>
-      <c r="E41" s="3" t="s">
-        <v>197</v>
-      </c>
-      <c r="F41" s="3" t="s">
-        <v>200</v>
-      </c>
-      <c r="G41" s="3" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
-        <v>81</v>
-      </c>
-      <c r="B42" t="s">
-        <v>83</v>
-      </c>
-      <c r="C42" t="s">
-        <v>255</v>
-      </c>
-      <c r="D42" s="4" t="s">
-        <v>430</v>
-      </c>
-      <c r="E42" t="s">
-        <v>199</v>
-      </c>
-      <c r="F42" t="s">
-        <v>201</v>
-      </c>
-      <c r="G42" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
-        <v>85</v>
-      </c>
-      <c r="B43" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="C43" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="D43" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="E43" s="3" t="s">
-        <v>171</v>
-      </c>
-      <c r="F43" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="G43" s="3" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
-        <v>86</v>
-      </c>
-      <c r="B44" t="s">
-        <v>84</v>
-      </c>
-      <c r="C44" t="s">
-        <v>256</v>
-      </c>
-      <c r="D44" t="s">
-        <v>284</v>
-      </c>
-      <c r="E44" s="4" t="s">
-        <v>405</v>
-      </c>
-      <c r="F44" t="s">
-        <v>202</v>
-      </c>
-      <c r="G44" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
-        <v>87</v>
-      </c>
-      <c r="B45" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="C45" s="3" t="s">
-        <v>206</v>
-      </c>
-      <c r="D45" s="3" t="s">
-        <v>285</v>
-      </c>
-      <c r="E45" s="4" t="s">
-        <v>406</v>
-      </c>
-      <c r="F45" s="3" t="s">
-        <v>342</v>
-      </c>
-      <c r="G45" s="3" t="s">
-        <v>374</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
-        <v>88</v>
-      </c>
-      <c r="B46" t="s">
-        <v>90</v>
-      </c>
-      <c r="C46" t="s">
-        <v>257</v>
-      </c>
-      <c r="D46" s="4" t="s">
-        <v>431</v>
-      </c>
-      <c r="E46" s="4" t="s">
-        <v>407</v>
-      </c>
-      <c r="F46" s="4" t="s">
+      <c r="E62" s="4" t="s">
+        <v>413</v>
+      </c>
+      <c r="F62" t="s">
+        <v>396</v>
+      </c>
+      <c r="G62" t="s">
+        <v>397</v>
+      </c>
+      <c r="H62" t="s">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A63" t="s">
+        <v>119</v>
+      </c>
+      <c r="B63" t="s">
+        <v>121</v>
+      </c>
+      <c r="C63" t="s">
+        <v>219</v>
+      </c>
+      <c r="D63" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="E63" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="F63" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="G63" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="H63" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A64" t="s">
+        <v>120</v>
+      </c>
+      <c r="B64" t="s">
+        <v>122</v>
+      </c>
+      <c r="C64" t="s">
+        <v>267</v>
+      </c>
+      <c r="D64" t="s">
+        <v>294</v>
+      </c>
+      <c r="E64" t="s">
+        <v>319</v>
+      </c>
+      <c r="F64" t="s">
+        <v>353</v>
+      </c>
+      <c r="G64" t="s">
+        <v>383</v>
+      </c>
+      <c r="H64" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A65" t="s">
+        <v>123</v>
+      </c>
+      <c r="B65" t="s">
+        <v>125</v>
+      </c>
+      <c r="C65" t="s">
+        <v>223</v>
+      </c>
+      <c r="D65" s="4" t="s">
+        <v>433</v>
+      </c>
+      <c r="E65" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="F65" s="3" t="s">
+        <v>354</v>
+      </c>
+      <c r="G65" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="H65" t="s">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A66" t="s">
+        <v>124</v>
+      </c>
+      <c r="B66" t="s">
+        <v>126</v>
+      </c>
+      <c r="C66" t="s">
+        <v>268</v>
+      </c>
+      <c r="D66" s="4" t="s">
+        <v>434</v>
+      </c>
+      <c r="E66" s="4" t="s">
+        <v>414</v>
+      </c>
+      <c r="F66" s="4" t="s">
         <v>441</v>
       </c>
-      <c r="G46" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>91</v>
-      </c>
-      <c r="B47" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="C47" s="3" t="s">
-        <v>258</v>
-      </c>
-      <c r="D47" s="3" t="s">
-        <v>286</v>
-      </c>
-      <c r="E47" s="4" t="s">
-        <v>408</v>
-      </c>
-      <c r="F47" s="3" t="s">
-        <v>207</v>
-      </c>
-      <c r="G47" s="3" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
-        <v>92</v>
-      </c>
-      <c r="B48" t="s">
-        <v>94</v>
-      </c>
-      <c r="C48" t="s">
-        <v>259</v>
-      </c>
-      <c r="D48" t="s">
-        <v>287</v>
-      </c>
-      <c r="E48" s="4" t="s">
-        <v>409</v>
-      </c>
-      <c r="F48" t="s">
-        <v>343</v>
-      </c>
-      <c r="G48" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
-        <v>95</v>
-      </c>
-      <c r="B49" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="C49" s="3" t="s">
-        <v>209</v>
-      </c>
-      <c r="D49" s="3" t="s">
-        <v>210</v>
-      </c>
-      <c r="E49" s="3" t="s">
-        <v>316</v>
-      </c>
-      <c r="F49" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="G49" s="3" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
-        <v>97</v>
-      </c>
-      <c r="B50" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="C50" s="3" t="s">
-        <v>260</v>
-      </c>
-      <c r="D50" s="3" t="s">
-        <v>288</v>
-      </c>
-      <c r="E50" s="4" t="s">
-        <v>418</v>
-      </c>
-      <c r="F50" s="3" t="s">
-        <v>212</v>
-      </c>
-      <c r="G50" s="3" t="s">
-        <v>377</v>
-      </c>
-    </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
-        <v>99</v>
-      </c>
-      <c r="B51" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="C51" s="3" t="s">
-        <v>214</v>
-      </c>
-      <c r="D51" s="3" t="s">
-        <v>289</v>
-      </c>
-      <c r="E51" s="4" t="s">
-        <v>410</v>
-      </c>
-      <c r="F51" s="3" t="s">
-        <v>344</v>
-      </c>
-      <c r="G51" s="3" t="s">
-        <v>378</v>
-      </c>
-    </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
-        <v>100</v>
-      </c>
-      <c r="B52" t="s">
-        <v>102</v>
-      </c>
-      <c r="C52" t="s">
-        <v>261</v>
-      </c>
-      <c r="D52" t="s">
-        <v>290</v>
-      </c>
-      <c r="E52" s="4" t="s">
-        <v>411</v>
-      </c>
-      <c r="F52" t="s">
-        <v>345</v>
-      </c>
-      <c r="G52" t="s">
-        <v>379</v>
-      </c>
-    </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
-        <v>103</v>
-      </c>
-      <c r="B53" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="C53" s="3" t="s">
-        <v>215</v>
-      </c>
-      <c r="D53" s="3" t="s">
-        <v>291</v>
-      </c>
-      <c r="E53" s="4" t="s">
-        <v>412</v>
-      </c>
-      <c r="F53" s="3" t="s">
-        <v>346</v>
-      </c>
-      <c r="G53" s="3" t="s">
-        <v>380</v>
-      </c>
-    </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A54" t="s">
-        <v>104</v>
-      </c>
-      <c r="B54" t="s">
-        <v>106</v>
-      </c>
-      <c r="C54" t="s">
-        <v>262</v>
-      </c>
-      <c r="D54" t="s">
-        <v>292</v>
-      </c>
-      <c r="E54" s="4" t="s">
-        <v>413</v>
-      </c>
-      <c r="F54" t="s">
-        <v>347</v>
-      </c>
-      <c r="G54" t="s">
-        <v>381</v>
-      </c>
-    </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
-        <v>109</v>
-      </c>
-      <c r="B55" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="C55" s="3" t="s">
-        <v>263</v>
-      </c>
-      <c r="D55" s="3" t="s">
-        <v>293</v>
-      </c>
-      <c r="E55" s="3" t="s">
-        <v>317</v>
-      </c>
-      <c r="F55" s="3" t="s">
-        <v>348</v>
-      </c>
-      <c r="G55" s="3" t="s">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A56" t="s">
-        <v>110</v>
-      </c>
-      <c r="B56" t="s">
-        <v>108</v>
-      </c>
-      <c r="C56" t="s">
-        <v>264</v>
-      </c>
-      <c r="D56" t="s">
-        <v>294</v>
-      </c>
-      <c r="E56" t="s">
-        <v>318</v>
-      </c>
-      <c r="F56" t="s">
-        <v>349</v>
-      </c>
-      <c r="G56" t="s">
-        <v>382</v>
-      </c>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A57" t="s">
-        <v>111</v>
-      </c>
-      <c r="B57" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="C57" s="3" t="s">
-        <v>265</v>
-      </c>
-      <c r="D57" s="4" t="s">
-        <v>432</v>
-      </c>
-      <c r="E57" s="3" t="s">
-        <v>319</v>
-      </c>
-      <c r="F57" s="3" t="s">
-        <v>216</v>
-      </c>
-      <c r="G57" s="3" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
-        <v>112</v>
-      </c>
-      <c r="B58" t="s">
-        <v>114</v>
-      </c>
-      <c r="C58" t="s">
-        <v>350</v>
-      </c>
-      <c r="D58" s="4" t="s">
-        <v>433</v>
-      </c>
-      <c r="E58" t="s">
-        <v>351</v>
-      </c>
-      <c r="F58" t="s">
-        <v>352</v>
-      </c>
-      <c r="G58" t="s">
-        <v>383</v>
-      </c>
-    </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
-        <v>115</v>
-      </c>
-      <c r="B59" t="s">
-        <v>117</v>
-      </c>
-      <c r="C59" t="s">
-        <v>217</v>
-      </c>
-      <c r="D59" t="s">
-        <v>396</v>
-      </c>
-      <c r="E59" t="s">
-        <v>218</v>
-      </c>
-      <c r="F59" t="s">
-        <v>353</v>
-      </c>
-      <c r="G59" t="s">
-        <v>399</v>
-      </c>
-    </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A60" t="s">
-        <v>116</v>
-      </c>
-      <c r="B60" t="s">
-        <v>118</v>
-      </c>
-      <c r="C60" t="s">
-        <v>266</v>
-      </c>
-      <c r="D60" t="s">
-        <v>395</v>
-      </c>
-      <c r="E60" s="4" t="s">
-        <v>414</v>
-      </c>
-      <c r="F60" t="s">
-        <v>397</v>
-      </c>
-      <c r="G60" t="s">
-        <v>398</v>
-      </c>
-    </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
-        <v>119</v>
-      </c>
-      <c r="B61" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="C61" s="3" t="s">
-        <v>219</v>
-      </c>
-      <c r="D61" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="E61" s="3" t="s">
-        <v>221</v>
-      </c>
-      <c r="F61" s="3" t="s">
-        <v>222</v>
-      </c>
-      <c r="G61" s="3" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
-        <v>120</v>
-      </c>
-      <c r="B62" t="s">
-        <v>122</v>
-      </c>
-      <c r="C62" t="s">
-        <v>267</v>
-      </c>
-      <c r="D62" t="s">
+      <c r="G66" t="s">
+        <v>384</v>
+      </c>
+      <c r="H66" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A67" t="s">
+        <v>127</v>
+      </c>
+      <c r="B67" t="s">
+        <v>129</v>
+      </c>
+      <c r="C67" t="s">
+        <v>224</v>
+      </c>
+      <c r="D67" s="4" t="s">
+        <v>435</v>
+      </c>
+      <c r="E67" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="F67" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="G67" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="H67" t="s">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A68" t="s">
+        <v>128</v>
+      </c>
+      <c r="B68" t="s">
+        <v>448</v>
+      </c>
+      <c r="C68" t="s">
+        <v>269</v>
+      </c>
+      <c r="D68" s="4" t="s">
+        <v>436</v>
+      </c>
+      <c r="E68" s="4" t="s">
+        <v>415</v>
+      </c>
+      <c r="F68" s="4" t="s">
+        <v>442</v>
+      </c>
+      <c r="G68" t="s">
+        <v>385</v>
+      </c>
+      <c r="H68" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A69" t="s">
+        <v>130</v>
+      </c>
+      <c r="B69" t="s">
+        <v>132</v>
+      </c>
+      <c r="C69" t="s">
+        <v>270</v>
+      </c>
+      <c r="D69" t="s">
         <v>295</v>
       </c>
-      <c r="E62" t="s">
+      <c r="E69" t="s">
         <v>320</v>
       </c>
-      <c r="F62" t="s">
-        <v>354</v>
-      </c>
-      <c r="G62" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
-        <v>123</v>
-      </c>
-      <c r="B63" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="C63" s="3" t="s">
-        <v>223</v>
-      </c>
-      <c r="D63" s="4" t="s">
-        <v>434</v>
-      </c>
-      <c r="E63" s="3" t="s">
-        <v>225</v>
-      </c>
-      <c r="F63" s="3" t="s">
+      <c r="F69" t="s">
         <v>355</v>
       </c>
-      <c r="G63" s="3" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A64" t="s">
-        <v>124</v>
-      </c>
-      <c r="B64" t="s">
-        <v>126</v>
-      </c>
-      <c r="C64" t="s">
-        <v>268</v>
-      </c>
-      <c r="D64" s="4" t="s">
-        <v>435</v>
-      </c>
-      <c r="E64" s="4" t="s">
-        <v>415</v>
-      </c>
-      <c r="F64" s="4" t="s">
-        <v>442</v>
-      </c>
-      <c r="G64" t="s">
-        <v>385</v>
-      </c>
-    </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A65" t="s">
-        <v>127</v>
-      </c>
-      <c r="B65" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="C65" s="3" t="s">
-        <v>224</v>
-      </c>
-      <c r="D65" s="4" t="s">
-        <v>436</v>
-      </c>
-      <c r="E65" s="3" t="s">
-        <v>226</v>
-      </c>
-      <c r="F65" s="3" t="s">
-        <v>228</v>
-      </c>
-      <c r="G65" s="3" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A66" t="s">
-        <v>128</v>
-      </c>
-      <c r="B66" t="s">
-        <v>270</v>
-      </c>
-      <c r="C66" t="s">
-        <v>269</v>
-      </c>
-      <c r="D66" s="4" t="s">
+      <c r="G69" t="s">
+        <v>386</v>
+      </c>
+      <c r="H69" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A70" t="s">
+        <v>131</v>
+      </c>
+      <c r="B70" t="s">
+        <v>133</v>
+      </c>
+      <c r="C70" t="s">
+        <v>271</v>
+      </c>
+      <c r="D70" t="s">
+        <v>296</v>
+      </c>
+      <c r="E70" t="s">
+        <v>321</v>
+      </c>
+      <c r="F70" t="s">
+        <v>356</v>
+      </c>
+      <c r="G70" t="s">
+        <v>387</v>
+      </c>
+      <c r="H70" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A71" t="s">
+        <v>134</v>
+      </c>
+      <c r="B71" t="s">
+        <v>136</v>
+      </c>
+      <c r="C71" t="s">
+        <v>272</v>
+      </c>
+      <c r="D71" s="4" t="s">
         <v>437</v>
       </c>
-      <c r="E66" s="4" t="s">
+      <c r="E71" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="F71" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="G71" s="3" t="s">
+        <v>388</v>
+      </c>
+      <c r="H71" t="s">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A72" t="s">
+        <v>135</v>
+      </c>
+      <c r="B72" t="s">
+        <v>137</v>
+      </c>
+      <c r="C72" t="s">
+        <v>273</v>
+      </c>
+      <c r="D72" s="4" t="s">
+        <v>438</v>
+      </c>
+      <c r="E72" s="4" t="s">
         <v>416</v>
       </c>
-      <c r="F66" s="4" t="s">
+      <c r="F72" s="4" t="s">
         <v>443</v>
       </c>
-      <c r="G66" t="s">
-        <v>386</v>
-      </c>
-    </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
-        <v>130</v>
-      </c>
-      <c r="B67" t="s">
-        <v>132</v>
-      </c>
-      <c r="C67" t="s">
-        <v>271</v>
-      </c>
-      <c r="D67" t="s">
-        <v>296</v>
-      </c>
-      <c r="E67" t="s">
-        <v>321</v>
-      </c>
-      <c r="F67" t="s">
-        <v>356</v>
-      </c>
-      <c r="G67" t="s">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
-        <v>131</v>
-      </c>
-      <c r="B68" t="s">
-        <v>133</v>
-      </c>
-      <c r="C68" t="s">
-        <v>272</v>
-      </c>
-      <c r="D68" t="s">
+      <c r="G72" t="s">
+        <v>389</v>
+      </c>
+      <c r="H72" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="73" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A73" t="s">
+        <v>138</v>
+      </c>
+      <c r="B73" t="s">
+        <v>140</v>
+      </c>
+      <c r="C73" t="s">
+        <v>232</v>
+      </c>
+      <c r="D73" s="3" t="s">
         <v>297</v>
       </c>
-      <c r="E68" t="s">
+      <c r="E73" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="F73" s="3" t="s">
+        <v>357</v>
+      </c>
+      <c r="G73" s="3" t="s">
+        <v>390</v>
+      </c>
+      <c r="H73" t="s">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="74" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A74" t="s">
+        <v>139</v>
+      </c>
+      <c r="B74" t="s">
+        <v>233</v>
+      </c>
+      <c r="C74" t="s">
+        <v>299</v>
+      </c>
+      <c r="D74" t="s">
+        <v>298</v>
+      </c>
+      <c r="E74" t="s">
         <v>322</v>
       </c>
-      <c r="F68" t="s">
-        <v>357</v>
-      </c>
-      <c r="G68" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A69" t="s">
-        <v>134</v>
-      </c>
-      <c r="B69" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="C69" s="3" t="s">
-        <v>273</v>
-      </c>
-      <c r="D69" s="4" t="s">
-        <v>438</v>
-      </c>
-      <c r="E69" s="3" t="s">
-        <v>227</v>
-      </c>
-      <c r="F69" s="3" t="s">
-        <v>229</v>
-      </c>
-      <c r="G69" s="3" t="s">
-        <v>389</v>
-      </c>
-    </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A70" t="s">
-        <v>135</v>
-      </c>
-      <c r="B70" t="s">
-        <v>137</v>
-      </c>
-      <c r="C70" t="s">
-        <v>274</v>
-      </c>
-      <c r="D70" s="4" t="s">
-        <v>439</v>
-      </c>
-      <c r="E70" s="4" t="s">
-        <v>417</v>
-      </c>
-      <c r="F70" s="4" t="s">
-        <v>444</v>
-      </c>
-      <c r="G70" t="s">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A71" t="s">
-        <v>138</v>
-      </c>
-      <c r="B71" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="C71" s="3" t="s">
-        <v>232</v>
-      </c>
-      <c r="D71" s="3" t="s">
-        <v>298</v>
-      </c>
-      <c r="E71" s="3" t="s">
-        <v>234</v>
-      </c>
-      <c r="F71" s="3" t="s">
+      <c r="F74" t="s">
         <v>358</v>
       </c>
-      <c r="G71" s="3" t="s">
+      <c r="G74" t="s">
         <v>391</v>
       </c>
-    </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A72" t="s">
-        <v>139</v>
-      </c>
-      <c r="B72" t="s">
-        <v>233</v>
-      </c>
-      <c r="C72" t="s">
-        <v>300</v>
-      </c>
-      <c r="D72" t="s">
-        <v>299</v>
-      </c>
-      <c r="E72" t="s">
-        <v>323</v>
-      </c>
-      <c r="F72" t="s">
-        <v>359</v>
-      </c>
-      <c r="G72" t="s">
-        <v>392</v>
+      <c r="H74" t="s">
+        <v>514</v>
       </c>
     </row>
   </sheetData>

</xml_diff>